<commit_message>
Hormiga con 11 de vida: muere en 3 golpes de gomitas
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance.xlsx
+++ b/balance.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="903">
   <si>
     <t>Balance de Junked Metal. Esta planilla se genera desde src/balance.json (npm run balance:xlsx) y vuelve al juego con npm run balance:import.</t>
   </si>
@@ -2120,6 +2120,18 @@
     <t>Un jefe pasa a fase 2 con menos de esta fracción de su vida</t>
   </si>
   <si>
+    <t>segunda_barra_vida</t>
+  </si>
+  <si>
+    <t>Jefe final: al vaciar la primera barra ruge y se llena una segunda con esta fracción de su vida</t>
+  </si>
+  <si>
+    <t>segunda_barra_dano</t>
+  </si>
+  <si>
+    <t>Jefe final en la segunda barra: multiplicador del daño que hace al auto</t>
+  </si>
+  <si>
     <t>fase2_vel</t>
   </si>
   <si>
@@ -2676,6 +2688,9 @@
   </si>
   <si>
     <t>Presencia: fracción del tiempo en que el equipo logra pegarle al jefe (0 a 1)</t>
+  </si>
+  <si>
+    <t>vida (con segunda barra)</t>
   </si>
   <si>
     <t>DPS supuesto del equipo</t>
@@ -4516,7 +4531,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" style="1" customWidth="1"/>
@@ -4584,7 +4599,7 @@
         <v>698</v>
       </c>
       <c r="B6">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="C6" t="s">
         <v>699</v>
@@ -4595,7 +4610,7 @@
         <v>700</v>
       </c>
       <c r="B7">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="C7" t="s">
         <v>701</v>
@@ -4606,7 +4621,7 @@
         <v>702</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>1.2</v>
       </c>
       <c r="C8" t="s">
         <v>703</v>
@@ -4617,7 +4632,7 @@
         <v>704</v>
       </c>
       <c r="B9">
-        <v>16</v>
+        <v>1.7</v>
       </c>
       <c r="C9" t="s">
         <v>705</v>
@@ -4628,7 +4643,7 @@
         <v>706</v>
       </c>
       <c r="B10">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
         <v>707</v>
@@ -4639,7 +4654,7 @@
         <v>708</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
         <v>709</v>
@@ -4650,7 +4665,7 @@
         <v>710</v>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
         <v>711</v>
@@ -4661,7 +4676,7 @@
         <v>712</v>
       </c>
       <c r="B13">
-        <v>1.2</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
         <v>713</v>
@@ -4672,7 +4687,7 @@
         <v>714</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C14" t="s">
         <v>715</v>
@@ -4683,7 +4698,7 @@
         <v>716</v>
       </c>
       <c r="B15">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="C15" t="s">
         <v>717</v>
@@ -4694,7 +4709,7 @@
         <v>718</v>
       </c>
       <c r="B16">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
         <v>719</v>
@@ -4705,7 +4720,7 @@
         <v>720</v>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>2.6</v>
       </c>
       <c r="C17" t="s">
         <v>721</v>
@@ -4716,7 +4731,7 @@
         <v>722</v>
       </c>
       <c r="B18">
-        <v>2.6</v>
+        <v>1.4</v>
       </c>
       <c r="C18" t="s">
         <v>723</v>
@@ -4727,7 +4742,7 @@
         <v>724</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
         <v>725</v>
@@ -4738,7 +4753,7 @@
         <v>726</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="C20" t="s">
         <v>727</v>
@@ -4749,7 +4764,7 @@
         <v>728</v>
       </c>
       <c r="B21">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="C21" t="s">
         <v>729</v>
@@ -4760,7 +4775,7 @@
         <v>730</v>
       </c>
       <c r="B22">
-        <v>1.7</v>
+        <v>3</v>
       </c>
       <c r="C22" t="s">
         <v>731</v>
@@ -4771,7 +4786,7 @@
         <v>732</v>
       </c>
       <c r="B23">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="C23" t="s">
         <v>733</v>
@@ -4782,7 +4797,7 @@
         <v>734</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>1.7</v>
       </c>
       <c r="C24" t="s">
         <v>735</v>
@@ -4793,7 +4808,7 @@
         <v>736</v>
       </c>
       <c r="B25">
-        <v>3</v>
+        <v>0.7</v>
       </c>
       <c r="C25" t="s">
         <v>737</v>
@@ -4804,7 +4819,7 @@
         <v>738</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C26" t="s">
         <v>739</v>
@@ -4815,7 +4830,7 @@
         <v>740</v>
       </c>
       <c r="B27">
-        <v>1.1</v>
+        <v>3</v>
       </c>
       <c r="C27" t="s">
         <v>741</v>
@@ -4826,7 +4841,7 @@
         <v>742</v>
       </c>
       <c r="B28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
         <v>743</v>
@@ -4837,7 +4852,7 @@
         <v>744</v>
       </c>
       <c r="B29">
-        <v>0.16</v>
+        <v>1.1</v>
       </c>
       <c r="C29" t="s">
         <v>745</v>
@@ -4848,7 +4863,7 @@
         <v>746</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C30" t="s">
         <v>747</v>
@@ -4859,7 +4874,7 @@
         <v>748</v>
       </c>
       <c r="B31">
-        <v>1.3</v>
+        <v>0.16</v>
       </c>
       <c r="C31" t="s">
         <v>749</v>
@@ -4870,7 +4885,7 @@
         <v>750</v>
       </c>
       <c r="B32">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C32" t="s">
         <v>751</v>
@@ -4881,7 +4896,7 @@
         <v>752</v>
       </c>
       <c r="B33">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="C33" t="s">
         <v>753</v>
@@ -4892,7 +4907,7 @@
         <v>754</v>
       </c>
       <c r="B34">
-        <v>0.5</v>
+        <v>22</v>
       </c>
       <c r="C34" t="s">
         <v>755</v>
@@ -4903,7 +4918,7 @@
         <v>756</v>
       </c>
       <c r="B35">
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="C35" t="s">
         <v>757</v>
@@ -4914,7 +4929,7 @@
         <v>758</v>
       </c>
       <c r="B36">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="C36" t="s">
         <v>759</v>
@@ -4925,7 +4940,7 @@
         <v>760</v>
       </c>
       <c r="B37">
-        <v>2.6</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
         <v>761</v>
@@ -4936,7 +4951,7 @@
         <v>762</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="C38" t="s">
         <v>763</v>
@@ -4947,7 +4962,7 @@
         <v>764</v>
       </c>
       <c r="B39">
-        <v>9</v>
+        <v>2.6</v>
       </c>
       <c r="C39" t="s">
         <v>765</v>
@@ -4958,7 +4973,7 @@
         <v>766</v>
       </c>
       <c r="B40">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C40" t="s">
         <v>767</v>
@@ -4969,7 +4984,7 @@
         <v>768</v>
       </c>
       <c r="B41">
-        <v>0.8</v>
+        <v>9</v>
       </c>
       <c r="C41" t="s">
         <v>769</v>
@@ -4980,7 +4995,7 @@
         <v>770</v>
       </c>
       <c r="B42">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C42" t="s">
         <v>771</v>
@@ -4991,7 +5006,7 @@
         <v>772</v>
       </c>
       <c r="B43">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="C43" t="s">
         <v>773</v>
@@ -5002,7 +5017,7 @@
         <v>774</v>
       </c>
       <c r="B44">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C44" t="s">
         <v>775</v>
@@ -5013,7 +5028,7 @@
         <v>776</v>
       </c>
       <c r="B45">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C45" t="s">
         <v>777</v>
@@ -5024,7 +5039,7 @@
         <v>778</v>
       </c>
       <c r="B46">
-        <v>3.5</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
         <v>779</v>
@@ -5035,7 +5050,7 @@
         <v>780</v>
       </c>
       <c r="B47">
-        <v>16</v>
+        <v>0.2</v>
       </c>
       <c r="C47" t="s">
         <v>781</v>
@@ -5046,7 +5061,7 @@
         <v>782</v>
       </c>
       <c r="B48">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="C48" t="s">
         <v>783</v>
@@ -5057,7 +5072,7 @@
         <v>784</v>
       </c>
       <c r="B49">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C49" t="s">
         <v>785</v>
@@ -5068,7 +5083,7 @@
         <v>786</v>
       </c>
       <c r="B50">
-        <v>2.2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="s">
         <v>787</v>
@@ -5079,7 +5094,7 @@
         <v>788</v>
       </c>
       <c r="B51">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
         <v>789</v>
@@ -5090,7 +5105,7 @@
         <v>790</v>
       </c>
       <c r="B52">
-        <v>14</v>
+        <v>2.2</v>
       </c>
       <c r="C52" t="s">
         <v>791</v>
@@ -5101,7 +5116,7 @@
         <v>792</v>
       </c>
       <c r="B53">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C53" t="s">
         <v>793</v>
@@ -5112,7 +5127,7 @@
         <v>794</v>
       </c>
       <c r="B54">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C54" t="s">
         <v>795</v>
@@ -5123,7 +5138,7 @@
         <v>796</v>
       </c>
       <c r="B55">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C55" t="s">
         <v>797</v>
@@ -5134,7 +5149,7 @@
         <v>798</v>
       </c>
       <c r="B56">
-        <v>0.5</v>
+        <v>28</v>
       </c>
       <c r="C56" t="s">
         <v>799</v>
@@ -5145,7 +5160,7 @@
         <v>800</v>
       </c>
       <c r="B57">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C57" t="s">
         <v>801</v>
@@ -5156,7 +5171,7 @@
         <v>802</v>
       </c>
       <c r="B58">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="C58" t="s">
         <v>803</v>
@@ -5167,7 +5182,7 @@
         <v>804</v>
       </c>
       <c r="B59">
-        <v>0.35</v>
+        <v>45</v>
       </c>
       <c r="C59" t="s">
         <v>805</v>
@@ -5178,7 +5193,7 @@
         <v>806</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="C60" t="s">
         <v>807</v>
@@ -5189,7 +5204,7 @@
         <v>808</v>
       </c>
       <c r="B61">
-        <v>24</v>
+        <v>0.35</v>
       </c>
       <c r="C61" t="s">
         <v>809</v>
@@ -5200,7 +5215,7 @@
         <v>810</v>
       </c>
       <c r="B62">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="C62" t="s">
         <v>811</v>
@@ -5211,7 +5226,7 @@
         <v>812</v>
       </c>
       <c r="B63">
-        <v>0.6</v>
+        <v>24</v>
       </c>
       <c r="C63" t="s">
         <v>813</v>
@@ -5222,7 +5237,7 @@
         <v>814</v>
       </c>
       <c r="B64">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="C64" t="s">
         <v>815</v>
@@ -5233,7 +5248,7 @@
         <v>816</v>
       </c>
       <c r="B65">
-        <v>17</v>
+        <v>0.6</v>
       </c>
       <c r="C65" t="s">
         <v>817</v>
@@ -5244,7 +5259,7 @@
         <v>818</v>
       </c>
       <c r="B66">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="C66" t="s">
         <v>819</v>
@@ -5255,7 +5270,7 @@
         <v>820</v>
       </c>
       <c r="B67">
-        <v>1.5</v>
+        <v>17</v>
       </c>
       <c r="C67" t="s">
         <v>821</v>
@@ -5266,7 +5281,7 @@
         <v>822</v>
       </c>
       <c r="B68">
-        <v>0.55</v>
+        <v>1.5</v>
       </c>
       <c r="C68" t="s">
         <v>823</v>
@@ -5277,7 +5292,7 @@
         <v>824</v>
       </c>
       <c r="B69">
-        <v>26</v>
+        <v>1.5</v>
       </c>
       <c r="C69" t="s">
         <v>825</v>
@@ -5288,7 +5303,7 @@
         <v>826</v>
       </c>
       <c r="B70">
-        <v>1.2</v>
+        <v>0.55</v>
       </c>
       <c r="C70" t="s">
         <v>827</v>
@@ -5299,7 +5314,7 @@
         <v>828</v>
       </c>
       <c r="B71">
-        <v>1.5</v>
+        <v>26</v>
       </c>
       <c r="C71" t="s">
         <v>829</v>
@@ -5310,7 +5325,7 @@
         <v>830</v>
       </c>
       <c r="B72">
-        <v>10</v>
+        <v>1.2</v>
       </c>
       <c r="C72" t="s">
         <v>831</v>
@@ -5321,7 +5336,7 @@
         <v>832</v>
       </c>
       <c r="B73">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="C73" t="s">
         <v>833</v>
@@ -5332,7 +5347,7 @@
         <v>834</v>
       </c>
       <c r="B74">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C74" t="s">
         <v>835</v>
@@ -5343,7 +5358,7 @@
         <v>836</v>
       </c>
       <c r="B75">
-        <v>0.35</v>
+        <v>4</v>
       </c>
       <c r="C75" t="s">
         <v>837</v>
@@ -5354,7 +5369,7 @@
         <v>838</v>
       </c>
       <c r="B76">
-        <v>0.25</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
         <v>839</v>
@@ -5365,7 +5380,7 @@
         <v>840</v>
       </c>
       <c r="B77">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="C77" t="s">
         <v>841</v>
@@ -5376,7 +5391,7 @@
         <v>842</v>
       </c>
       <c r="B78">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="C78" t="s">
         <v>843</v>
@@ -5387,7 +5402,7 @@
         <v>844</v>
       </c>
       <c r="B79">
-        <v>3.8</v>
+        <v>0.25</v>
       </c>
       <c r="C79" t="s">
         <v>845</v>
@@ -5398,7 +5413,7 @@
         <v>846</v>
       </c>
       <c r="B80">
-        <v>2.6</v>
+        <v>25</v>
       </c>
       <c r="C80" t="s">
         <v>847</v>
@@ -5409,7 +5424,7 @@
         <v>848</v>
       </c>
       <c r="B81">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="C81" t="s">
         <v>849</v>
@@ -5420,7 +5435,7 @@
         <v>850</v>
       </c>
       <c r="B82">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="C82" t="s">
         <v>851</v>
@@ -5431,7 +5446,7 @@
         <v>852</v>
       </c>
       <c r="B83">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="C83" t="s">
         <v>853</v>
@@ -5442,7 +5457,7 @@
         <v>854</v>
       </c>
       <c r="B84">
-        <v>1.2</v>
+        <v>2.1</v>
       </c>
       <c r="C84" t="s">
         <v>855</v>
@@ -5453,7 +5468,7 @@
         <v>856</v>
       </c>
       <c r="B85">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="C85" t="s">
         <v>857</v>
@@ -5464,32 +5479,32 @@
         <v>858</v>
       </c>
       <c r="B86">
-        <v>0.75</v>
+        <v>1.2</v>
       </c>
       <c r="C86" t="s">
-        <v>847</v>
+        <v>859</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B87">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B88">
-        <v>26</v>
+        <v>0.75</v>
       </c>
       <c r="C88" t="s">
-        <v>862</v>
+        <v>851</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -5497,7 +5512,7 @@
         <v>863</v>
       </c>
       <c r="B89">
-        <v>2.6</v>
+        <v>30</v>
       </c>
       <c r="C89" t="s">
         <v>864</v>
@@ -5508,7 +5523,7 @@
         <v>865</v>
       </c>
       <c r="B90">
-        <v>0.9</v>
+        <v>26</v>
       </c>
       <c r="C90" t="s">
         <v>866</v>
@@ -5519,10 +5534,32 @@
         <v>867</v>
       </c>
       <c r="B91">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="C91" t="s">
         <v>868</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="B92">
+        <v>0.9</v>
+      </c>
+      <c r="C92" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>871</v>
+      </c>
+      <c r="B93">
+        <v>1.4</v>
+      </c>
+      <c r="C93" t="s">
+        <v>872</v>
       </c>
     </row>
   </sheetData>
@@ -5545,17 +5582,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="B4" s="7">
         <v>0</v>
@@ -5563,7 +5600,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="B5" s="7">
         <v>1</v>
@@ -5571,7 +5608,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>177</v>
@@ -5579,7 +5616,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="B7" s="7">
         <v>12</v>
@@ -5587,7 +5624,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="B8" s="7">
         <v>1</v>
@@ -5595,7 +5632,7 @@
     </row>
     <row r="9" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D9" s="8" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="E9" s="8">
         <f>INDEX(armas!$B$3:$B$500,MATCH(E$10,armas!$A$3:$A$500,0))</f>
@@ -5670,12 +5707,12 @@
         <f>INDEX(armas!$B$3:$B$500,MATCH(AB$10,armas!$A$3:$A$500,0))</f>
       </c>
       <c r="AC9" s="8" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
     <row r="10" spans="4:29" x14ac:dyDescent="0.25">
       <c r="D10" s="9" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>105</v>
@@ -5755,7 +5792,7 @@
     </row>
     <row r="11" spans="4:28" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -5841,7 +5878,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="E12" s="10">
         <f>(INDEX(armas!$D$3:$D$500,MATCH(E$10,armas!$A$3:$A$500,0))+INDEX(armas!$E$3:$E$500,MATCH(E$10,armas!$A$3:$A$500,0))*E$11)*$B$5</f>
@@ -7097,17 +7134,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="B4" s="7">
         <v>0.8</v>
@@ -7124,16 +7161,16 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>9</v>
+        <v>888</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -7147,7 +7184,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A7,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D7">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A7,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A7,enemigos!$A$3:$A$500,0))*IF($C7="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E7" s="7">
         <v>200</v>
@@ -7170,7 +7207,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A8,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D8">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A8,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A8,enemigos!$A$3:$A$500,0))*IF($C8="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E8" s="7">
         <v>200</v>
@@ -7193,7 +7230,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A9,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D9">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A9,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A9,enemigos!$A$3:$A$500,0))*IF($C9="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E9" s="7">
         <v>200</v>
@@ -7216,7 +7253,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A10,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D10">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A10,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A10,enemigos!$A$3:$A$500,0))*IF($C10="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E10" s="7">
         <v>200</v>
@@ -7239,7 +7276,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A11,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D11">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A11,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A11,enemigos!$A$3:$A$500,0))*IF($C11="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E11" s="7">
         <v>600</v>
@@ -7262,7 +7299,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A12,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D12">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A12,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A12,enemigos!$A$3:$A$500,0))*IF($C12="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E12" s="7">
         <v>600</v>
@@ -7285,7 +7322,7 @@
         <f>INDEX(enemigos!$C$3:$C$500,MATCH($A13,enemigos!$A$3:$A$500,0))</f>
       </c>
       <c r="D13">
-        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A13,enemigos!$A$3:$A$500,0))</f>
+        <f>INDEX(enemigos!$D$3:$D$500,MATCH($A13,enemigos!$A$3:$A$500,0))*IF($C13="jefe_final",1+INDEX(ataques!$B$3:$B$500,MATCH("segunda_barra_vida",ataques!$A$3:$A$500,0)),1)</f>
       </c>
       <c r="E13" s="7">
         <v>600</v>
@@ -7315,17 +7352,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B4" s="7">
         <v>100</v>
@@ -7333,7 +7370,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="B5" s="7">
         <v>420</v>
@@ -7341,7 +7378,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="B6" s="7">
         <v>600</v>
@@ -7349,7 +7386,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="B7" s="7">
         <v>1</v>
@@ -7357,7 +7394,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="B8">
         <f>INT((B7*INDEX(ritmo!$B$3:$B$500,MATCH("tornillos_jefe",ritmo!$A$3:$A$500,0))+INT(B5/INDEX(ritmo!$B$3:$B$500,MATCH("tornillos_div_tiempo",ritmo!$A$3:$A$500,0)))+INT(B6*INDEX(ritmo!$B$3:$B$500,MATCH("dureza_xp",ritmo!$A$3:$A$500,0))/INDEX(ritmo!$B$3:$B$500,MATCH("tornillos_div_bajas",ritmo!$A$3:$A$500,0)))))</f>
@@ -7404,7 +7441,7 @@
         <v>233</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -8333,7 +8370,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B32" t="s">
         <v>177</v>
@@ -8350,7 +8387,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B33" t="s">
         <v>179</v>
@@ -8367,7 +8404,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B34" t="s">
         <v>181</v>
@@ -8384,7 +8421,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B35" t="s">
         <v>183</v>
@@ -8401,7 +8438,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B36" t="s">
         <v>185</v>
@@ -8418,7 +8455,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B37" t="s">
         <v>186</v>
@@ -8435,7 +8472,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B38" t="s">
         <v>133</v>
@@ -8452,7 +8489,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B39" t="s">
         <v>189</v>
@@ -8469,7 +8506,7 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B40" t="s">
         <v>214</v>
@@ -8486,7 +8523,7 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B41" t="s">
         <v>216</v>
@@ -8503,7 +8540,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B42" t="s">
         <v>35</v>
@@ -8520,7 +8557,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B43" t="s">
         <v>219</v>
@@ -8537,7 +8574,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B44" t="s">
         <v>221</v>
@@ -8554,7 +8591,7 @@
     </row>
     <row r="46" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C46" s="1" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="N46" s="11">
         <f>SUM(N11:N44)</f>
@@ -8657,7 +8694,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>8</v>
@@ -9007,7 +9044,7 @@
         <v>52</v>
       </c>
       <c r="D13">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="E13">
         <v>9</v>
@@ -9042,7 +9079,7 @@
         <v>52</v>
       </c>
       <c r="D14">
-        <v>40000</v>
+        <v>7500</v>
       </c>
       <c r="E14">
         <v>7</v>
@@ -9077,7 +9114,7 @@
         <v>52</v>
       </c>
       <c r="D15">
-        <v>30000</v>
+        <v>7000</v>
       </c>
       <c r="E15">
         <v>8</v>

</xml_diff>

<commit_message>
Autos y pilotos con apodos y una frase que explica el nombre
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance.xlsx
+++ b/balance.xlsx
@@ -566,40 +566,40 @@
     <t>monster</t>
   </si>
   <si>
-    <t>Crisis de los 40</t>
+    <t>El Loco Cuarentón</t>
   </si>
   <si>
     <t>formula</t>
   </si>
   <si>
-    <t>Multa Pendiente</t>
+    <t>El Apurado</t>
   </si>
   <si>
     <t>tanque</t>
   </si>
   <si>
-    <t>Política Exterior</t>
+    <t>El Suegro</t>
   </si>
   <si>
     <t>carrera</t>
   </si>
   <si>
-    <t>Sin Seguro</t>
+    <t>El Sin Seguro</t>
   </si>
   <si>
     <t>axel</t>
   </si>
   <si>
-    <t>Axel Sin Licencia</t>
-  </si>
-  <si>
-    <t>Diabetes Tipo Turbo</t>
+    <t>El Sin Licencia</t>
+  </si>
+  <si>
+    <t>El Tío del Helado</t>
   </si>
   <si>
     <t>combi</t>
   </si>
   <si>
-    <t>La Combi del Tío Raro</t>
+    <t>El Tío Raro</t>
   </si>
   <si>
     <t>dano_mult</t>
@@ -674,28 +674,28 @@
     <t>soldadito</t>
   </si>
   <si>
-    <t>Sargento Sin Pensión</t>
+    <t>El Sargento Sin Pensión</t>
   </si>
   <si>
     <t>muneca</t>
   </si>
   <si>
-    <t>Doña Trapo, Divorciada</t>
-  </si>
-  <si>
-    <t>Robot en Crisis Existencial</t>
+    <t>La Divorciada de Trapo</t>
+  </si>
+  <si>
+    <t>El Robot en Crisis</t>
   </si>
   <si>
     <t>dino</t>
   </si>
   <si>
-    <t>Rex, Ya No Tan Temible</t>
+    <t>El Rex Jubilado</t>
   </si>
   <si>
     <t>figura</t>
   </si>
   <si>
-    <t>Mega Macho Sin Articulaciones</t>
+    <t>El Mega Macho</t>
   </si>
   <si>
     <t>efecto</t>

</xml_diff>